<commit_message>
test(attendance): ensure mock class status is InProgress for attendance operations
</commit_message>
<xml_diff>
--- a/Report/Demo_Bulk_Import_Classes_Roster.xlsx
+++ b/Report/Demo_Bulk_Import_Classes_Roster.xlsx
@@ -546,12 +546,12 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>31/12/2026</t>
+          <t>15/01/2027</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">

</xml_diff>